<commit_message>
feat : PVD-demo machine
</commit_message>
<xml_diff>
--- a/data/input/PVD_FMEA.xlsx
+++ b/data/input/PVD_FMEA.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="81">
   <si>
     <t>設計製程項目
 (Process Design)</t>
@@ -364,6 +364,39 @@
   <si>
     <t>電路阻抗不符合設計值</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>machine_action</t>
+  </si>
+  <si>
+    <t>{"machine_id":"PVD-DEMO-01","setpoints":{"button_1":10,"button_2":20,"button_3":30}}</t>
+  </si>
+  <si>
+    <t>{"machine_id":"PVD-DEMO-01","setpoints":{"button_1":15,"button_2":25,"button_3":35}}</t>
+  </si>
+  <si>
+    <t>{"machine_id":"PVD-DEMO-01","setpoints":{"button_1":20,"button_2":30,"button_3":40}}</t>
+  </si>
+  <si>
+    <t>{"machine_id":"PVD-DEMO-01","setpoints":{"button_1":25,"button_2":35,"button_3":45}}</t>
+  </si>
+  <si>
+    <t>{"machine_id":"PVD-DEMO-01","setpoints":{"button_1":30,"button_2":40,"button_3":50}}</t>
+  </si>
+  <si>
+    <t>{"machine_id":"PVD-DEMO-01","setpoints":{"button_1":35,"button_2":45,"button_3":55}}</t>
+  </si>
+  <si>
+    <t>{"machine_id":"PVD-DEMO-01","setpoints":{"button_1":40,"button_2":50,"button_3":60}}</t>
+  </si>
+  <si>
+    <t>{"machine_id":"PVD-DEMO-01","setpoints":{"button_1":45,"button_2":55,"button_3":65}}</t>
+  </si>
+  <si>
+    <t>{"machine_id":"PVD-DEMO-01","setpoints":{"button_1":50,"button_2":60,"button_3":70}}</t>
+  </si>
+  <si>
+    <t>{"machine_id":"PVD-DEMO-01","setpoints":{"button_1":55,"button_2":65,"button_3":75}}</t>
   </si>
 </sst>
 </file>
@@ -1044,6 +1077,9 @@
       <c r="S2" s="11" t="s">
         <v>11</v>
       </c>
+      <c r="T2" s="11" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="3" spans="2:20" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1"/>
@@ -1099,7 +1135,9 @@
         <v>32</v>
       </c>
       <c r="S3" s="11"/>
-      <c r="T3" s="6"/>
+      <c r="T3" s="2" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="4" spans="2:20" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="1"/>
@@ -1154,7 +1192,7 @@
       </c>
       <c r="S4" s="11"/>
       <c r="T4" s="2" t="s">
-        <v>25</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" spans="2:20" s="8" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -1209,7 +1247,9 @@
         <v>120</v>
       </c>
       <c r="S5" s="11"/>
-      <c r="T5" s="2"/>
+      <c r="T5" s="2" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="6" spans="2:20" s="8" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="7"/>
@@ -1263,7 +1303,9 @@
         <v>48</v>
       </c>
       <c r="S6" s="11"/>
-      <c r="T6" s="2"/>
+      <c r="T6" s="2" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="7" spans="2:20" ht="85.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="1"/>
@@ -1319,6 +1361,9 @@
         <v>63</v>
       </c>
       <c r="S7" s="11"/>
+      <c r="T7" s="2" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="8" spans="2:20" s="8" customFormat="1" ht="81.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="7"/>
@@ -1372,6 +1417,9 @@
         <v>54</v>
       </c>
       <c r="S8" s="11"/>
+      <c r="T8" s="2" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="9" spans="2:20" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="1"/>
@@ -1425,6 +1473,9 @@
         <v>54</v>
       </c>
       <c r="S9" s="11"/>
+      <c r="T9" s="2" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="10" spans="2:20" ht="131.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="1"/>
@@ -1478,6 +1529,9 @@
         <v>120</v>
       </c>
       <c r="S10" s="11"/>
+      <c r="T10" s="2" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="11" spans="2:20" ht="75.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="1"/>
@@ -1531,6 +1585,9 @@
         <v>96</v>
       </c>
       <c r="S11" s="11"/>
+      <c r="T11" s="2" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="12" spans="2:20" ht="79.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="1"/>
@@ -1584,6 +1641,9 @@
         <v>200</v>
       </c>
       <c r="S12" s="11"/>
+      <c r="T12" s="2" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="13" spans="2:20" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E13" s="10"/>

</xml_diff>